<commit_message>
Agregado script de carga de datos y archivo Excel para poblar la BD
</commit_message>
<xml_diff>
--- a/datos_municipio.xlsx
+++ b/datos_municipio.xlsx
@@ -4,7 +4,7 @@
   <workbookPr date1904="0"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="4" showHorizontalScroll="1" showVerticalScroll="1"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0" showHorizontalScroll="1" showVerticalScroll="1"/>
   </bookViews>
   <sheets>
     <sheet name="localidades" sheetId="1" state="visible" r:id="rId1"/>
@@ -18751,7 +18751,7 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">

</xml_diff>